<commit_message>
fixed the print prev ifor the mbformula
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/mb_formula_template.xlsx
+++ b/core/main/templates/print_excel/mb_formula_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\VS Code Web\ColorMatch\core\main\templates\print_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26917238-DC3D-4AB4-A71E-6F5EDB215888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8698093-1013-46CA-8695-BE66E90F31ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>EXTRUDER COLOR MATCHING FORM</t>
   </si>
@@ -79,9 +79,6 @@
   </si>
   <si>
     <t>Application :</t>
-  </si>
-  <si>
-    <t>__________________</t>
   </si>
   <si>
     <t>FM00006D</t>
@@ -211,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -225,20 +222,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -625,14 +621,14 @@
     <row r="2" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
       <c r="E4" s="3"/>
       <c r="F4" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G4" s="3"/>
     </row>
@@ -641,54 +637,54 @@
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="1"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="15"/>
       <c r="D6" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="16"/>
+      <c r="F6" s="10"/>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="1"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="18"/>
+      <c r="F7" s="12"/>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="1"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="16"/>
+      <c r="F8" s="14"/>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="1"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="18"/>
+        <v>19</v>
+      </c>
+      <c r="F9" s="12"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -696,15 +692,15 @@
     </row>
     <row r="10" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="B10" s="10"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E10" s="1"/>
-      <c r="F10" s="16"/>
+      <c r="F10" s="10"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -808,8 +804,8 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="1:6" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>6</v>
       </c>
@@ -822,9 +818,7 @@
       <c r="E24" t="s">
         <v>4</v>
       </c>
-      <c r="F24" t="s">
-        <v>18</v>
-      </c>
+      <c r="F24" s="12"/>
     </row>
     <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
@@ -840,10 +834,10 @@
       <c r="F29" s="6"/>
     </row>
     <row r="31" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A31" s="9"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
       <c r="E31" s="3"/>
       <c r="F31" s="7"/>
     </row>
@@ -877,150 +871,54 @@
       <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-    </row>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="12"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-    </row>
+      <c r="A37" s="4"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="13"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-    </row>
-    <row r="40" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="12"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-    </row>
-    <row r="41" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="12"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-      <c r="F41" s="12"/>
-    </row>
-    <row r="42" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="12"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-    </row>
-    <row r="43" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="12"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="12"/>
-    </row>
-    <row r="44" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="12"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-    </row>
-    <row r="45" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="12"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
-    </row>
-    <row r="46" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="12"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-    </row>
-    <row r="47" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="12"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-    </row>
-    <row r="48" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="12"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
-    </row>
-    <row r="49" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="12"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="12"/>
-      <c r="F49" s="12"/>
-    </row>
-    <row r="50" spans="1:6" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="12"/>
-      <c r="B50" s="12"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="12"/>
-    </row>
-    <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="14"/>
-      <c r="B51" s="15"/>
-      <c r="C51" s="12"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="12"/>
-      <c r="F51" s="12"/>
-    </row>
-    <row r="52" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="14"/>
-      <c r="B52" s="15"/>
-      <c r="C52" s="12"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="12"/>
-      <c r="F52" s="12"/>
-    </row>
-    <row r="53" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="12"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="12"/>
-      <c r="F53" s="12"/>
-    </row>
-    <row r="54" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="A39" s="9"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+    </row>
+    <row r="40" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="1:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="6"/>
+      <c r="B51" s="8"/>
+      <c r="D51" s="6"/>
+    </row>
+    <row r="52" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="6"/>
+      <c r="B52" s="8"/>
+    </row>
+    <row r="53" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="6"/>
+    </row>
+    <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A31:D31"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.7" right="0.7" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="5" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="10002" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
UPDATED THE MASTER FORMULA TEMPLATE
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/mb_formula_template.xlsx
+++ b/core/main/templates/print_excel/mb_formula_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\VS Code Web\ColorMatch\core\main\templates\print_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8698093-1013-46CA-8695-BE66E90F31ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980DF770-4DA3-4B0F-A265-9742DB667B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,14 +18,14 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$F$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$G$25</definedName>
   </definedNames>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>EXTRUDER COLOR MATCHING FORM</t>
   </si>
@@ -61,9 +61,6 @@
   </si>
   <si>
     <t>Total Weight</t>
-  </si>
-  <si>
-    <t>______________</t>
   </si>
   <si>
     <t>Date                :</t>
@@ -161,7 +158,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -204,11 +201,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -228,13 +251,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -262,7 +302,7 @@
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>514350</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
@@ -605,316 +645,353 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" customWidth="1"/>
-    <col min="5" max="5" width="1.28515625" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="11.85546875" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="3.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
+    <col min="6" max="6" width="1" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="13" t="s">
+    <row r="1" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:11" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G6" s="10"/>
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="4"/>
       <c r="C7" s="10"/>
-      <c r="D7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="12"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="10"/>
+      <c r="E7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="12"/>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="11"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="1" t="s">
+      <c r="D8" s="11"/>
+      <c r="E8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G8" s="13"/>
+      <c r="K8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="12"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="1"/>
+        <v>19</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="10"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
-    </row>
-    <row r="12" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="K10" s="1"/>
+    </row>
+    <row r="12" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="16"/>
+      <c r="C12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5" t="s">
+      <c r="E12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+    <row r="13" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="17"/>
+      <c r="B13" s="18"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="17"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="17"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="17"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="17"/>
+      <c r="B19" s="18"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
+      <c r="G19" s="2"/>
+    </row>
+    <row r="20" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="17"/>
+      <c r="B20" s="18"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="17"/>
+      <c r="B21" s="18"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="17"/>
+      <c r="B22" s="18"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-    </row>
-    <row r="23" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="E24" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>4</v>
       </c>
-      <c r="F24" s="12"/>
-    </row>
-    <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G24" s="12"/>
+    </row>
+    <row r="25" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F29" s="6"/>
-    </row>
-    <row r="31" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="7"/>
-    </row>
-    <row r="32" spans="1:6" ht="2.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+    </row>
+    <row r="26" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G29" s="6"/>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="7"/>
+    </row>
+    <row r="32" spans="1:7" ht="2.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
-      <c r="B33" s="1"/>
+      <c r="B33" s="4"/>
       <c r="C33" s="1"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="4"/>
       <c r="F33" s="1"/>
-    </row>
-    <row r="34" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G33" s="1"/>
+    </row>
+    <row r="34" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
-      <c r="B34" s="1"/>
+      <c r="B34" s="4"/>
       <c r="C34" s="1"/>
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D34" s="1"/>
+      <c r="E34" s="4"/>
+    </row>
+    <row r="35" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
-      <c r="B35" s="1"/>
+      <c r="B35" s="4"/>
       <c r="C35" s="1"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="4"/>
       <c r="F35" s="1"/>
-    </row>
-    <row r="36" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G35" s="1"/>
+    </row>
+    <row r="36" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
-      <c r="B36" s="1"/>
+      <c r="B36" s="4"/>
       <c r="C36" s="1"/>
-      <c r="D36" s="4"/>
-    </row>
-    <row r="37" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D36" s="1"/>
+      <c r="E36" s="4"/>
+    </row>
+    <row r="37" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
-      <c r="B37" s="1"/>
+      <c r="B37" s="4"/>
       <c r="C37" s="1"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="4"/>
       <c r="F37" s="1"/>
-    </row>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G37" s="1"/>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
-    </row>
-    <row r="40" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="1:5" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6"/>
-      <c r="B51" s="8"/>
-      <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="6"/>
+      <c r="C51" s="8"/>
+      <c r="E51" s="6"/>
+    </row>
+    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6"/>
-      <c r="B52" s="8"/>
-    </row>
-    <row r="53" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="6"/>
-    </row>
-    <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B52" s="6"/>
+      <c r="C52" s="8"/>
+    </row>
+    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="6"/>
+    </row>
+    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="A31:D31"/>
+  <mergeCells count="15">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
revert back to original  setup of print
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/mb_formula_template.xlsx
+++ b/core/main/templates/print_excel/mb_formula_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\VS Code Web\ColorMatch\core\main\templates\print_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980DF770-4DA3-4B0F-A265-9742DB667B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17E7D67-C432-4076-A2B4-B704E45DB93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -94,6 +94,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -231,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -273,6 +276,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -679,7 +685,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="C6" s="13"/>
+      <c r="C6" s="21"/>
       <c r="D6" s="10"/>
       <c r="E6" s="4" t="s">
         <v>2</v>

</xml_diff>